<commit_message>
feat(catalog): seo en importador excel, agrupacion de colores y footer version 3
</commit_message>
<xml_diff>
--- a/public/plantillas/plantilla_carga_productos_onestar.xlsx
+++ b/public/plantillas/plantilla_carga_productos_onestar.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA5"/>
+  <dimension ref="A1:AH5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -481,6 +481,27 @@
       <c r="AA1" t="str">
         <v>Producto listo</v>
       </c>
+      <c r="AB1" t="str">
+        <v>Grupo color</v>
+      </c>
+      <c r="AC1" t="str">
+        <v>¿Destacado?</v>
+      </c>
+      <c r="AD1" t="str">
+        <v>¿Lanzamiento?</v>
+      </c>
+      <c r="AE1" t="str">
+        <v>Beneficios</v>
+      </c>
+      <c r="AF1" t="str">
+        <v>Preguntas frecuentes</v>
+      </c>
+      <c r="AG1" t="str">
+        <v>Título SEO</v>
+      </c>
+      <c r="AH1" t="str">
+        <v>Descripción SEO</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -564,6 +585,27 @@
       <c r="AA2" t="str">
         <v>OK = listo para publicar | PENDIENTE = omitir</v>
       </c>
+      <c r="AB2" t="str">
+        <v>Nombre o código para agrupar colores del mismo modelo</v>
+      </c>
+      <c r="AC2" t="str">
+        <v>SI | NO</v>
+      </c>
+      <c r="AD2" t="str">
+        <v>SI | NO</v>
+      </c>
+      <c r="AE2" t="str">
+        <v>Beneficios separados por salto de línea o punto y coma</v>
+      </c>
+      <c r="AF2" t="str">
+        <v>Preguntas y respuestas en formato ¿Pregunta? | Respuesta</v>
+      </c>
+      <c r="AG2" t="str">
+        <v>Título para buscadores (recomendado hasta 60 caracteres)</v>
+      </c>
+      <c r="AH2" t="str">
+        <v>Descripción para buscadores (recomendado hasta 160 caracteres)</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -647,6 +689,27 @@
       <c r="AA3" t="str">
         <v>OK</v>
       </c>
+      <c r="AB3" t="str">
+        <v>Knu Skool</v>
+      </c>
+      <c r="AC3" t="str">
+        <v>NO</v>
+      </c>
+      <c r="AD3" t="str">
+        <v>NO</v>
+      </c>
+      <c r="AE3" t="str">
+        <v>Diseño acolchado;Suela waffle resistente</v>
+      </c>
+      <c r="AF3" t="str">
+        <v>¿Es original? | Sí, 100% original con garantía</v>
+      </c>
+      <c r="AG3" t="str">
+        <v>Tenis Vans Knu Skool Black White | One Star Colombia</v>
+      </c>
+      <c r="AH3" t="str">
+        <v>Compra tenis Vans Knu Skool Black White originales en One Star. Envíos a toda Colombia.</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -730,6 +793,27 @@
       <c r="AA4" t="str">
         <v>OK</v>
       </c>
+      <c r="AB4" t="str">
+        <v>Knu Skool</v>
+      </c>
+      <c r="AC4" t="str">
+        <v>NO</v>
+      </c>
+      <c r="AD4" t="str">
+        <v>NO</v>
+      </c>
+      <c r="AE4" t="str">
+        <v>Diseño acolchado;Suela waffle resistente</v>
+      </c>
+      <c r="AF4" t="str">
+        <v>¿Es original? | Sí, 100% original con garantía</v>
+      </c>
+      <c r="AG4" t="str">
+        <v>Tenis Vans Knu Skool Black White | One Star Colombia</v>
+      </c>
+      <c r="AH4" t="str">
+        <v>Compra tenis Vans Knu Skool Black White originales en One Star. Envíos a toda Colombia.</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -813,10 +897,31 @@
       <c r="AA5" t="str">
         <v>OK</v>
       </c>
+      <c r="AB5" t="str">
+        <v>Knu Skool</v>
+      </c>
+      <c r="AC5" t="str">
+        <v>NO</v>
+      </c>
+      <c r="AD5" t="str">
+        <v>NO</v>
+      </c>
+      <c r="AE5" t="str">
+        <v>Diseño acolchado;Suela waffle resistente</v>
+      </c>
+      <c r="AF5" t="str">
+        <v>¿Es original? | Sí, 100% original con garantía</v>
+      </c>
+      <c r="AG5" t="str">
+        <v>Tenis Vans Knu Skool Black White | One Star Colombia</v>
+      </c>
+      <c r="AH5" t="str">
+        <v>Compra tenis Vans Knu Skool Black White originales en One Star. Envíos a toda Colombia.</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AA5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
wip(importador): columna Ventas cruzadas en el Excel (sin pruebas aún)
- Columna "Ventas cruzadas" (alias: VENTA CRUZADA, COMBÍNALO CON, crossSells):
  referencias SKU o código base separadas por coma, máx. 12.
- Al aplicar: conecta Product.crossSells al final de la transacción
  (sirve con productos del mismo archivo). Celda vacía = no toca nada.
- Vista previa: aviso "ventas cruzadas sin producto: X".
- Plantilla .xlsx con la columna nueva.
Falta: pruebas (lib/cross-sell, vista previa, apply) y probar en local.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantillas/plantilla_carga_productos_onestar.xlsx
+++ b/public/plantillas/plantilla_carga_productos_onestar.xlsx
@@ -121,10 +121,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -156,10 +156,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH5"/>
+  <dimension ref="A1:AI5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -502,6 +502,9 @@
       <c r="AH1" t="str">
         <v>Descripción SEO</v>
       </c>
+      <c r="AI1" t="str">
+        <v>Ventas cruzadas</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -606,6 +609,9 @@
       <c r="AH2" t="str">
         <v>Descripción para buscadores (recomendado hasta 160 caracteres)</v>
       </c>
+      <c r="AI2" t="str">
+        <v>Referencias de productos para sugerir con este (SKU o código base), separadas por coma. Ej: MEDIAS-TRAIL, LIMPIADOR-01</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -710,6 +716,9 @@
       <c r="AH3" t="str">
         <v>Compra tenis Vans Knu Skool Black White originales en One Star. Envíos a toda Colombia.</v>
       </c>
+      <c r="AI3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -814,6 +823,9 @@
       <c r="AH4" t="str">
         <v>Compra tenis Vans Knu Skool Black White originales en One Star. Envíos a toda Colombia.</v>
       </c>
+      <c r="AI4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -918,10 +930,13 @@
       <c r="AH5" t="str">
         <v>Compra tenis Vans Knu Skool Black White originales en One Star. Envíos a toda Colombia.</v>
       </c>
+      <c r="AI5" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AI5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>